<commit_message>
modified:   1/app/logs/execution.log 	modified:   1/app/output/ground_truth.xlsx 	modified:   1/app/output/harness_log.csv
</commit_message>
<xml_diff>
--- a/1/app/output/ground_truth.xlsx
+++ b/1/app/output/ground_truth.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Economic analysis of knowledge‑intensive industries\1\app\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A274BB37-0EB4-4D28-98B8-A78B62C679C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF39CD3E-8BC3-44A4-A9F0-6522EE54529B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3624" yWindow="3624" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -565,7 +565,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-09-14T08:10:52.014831+00:00</t>
+    <t>2026-09-14T08:16:12.931028+00:00</t>
   </si>
   <si>
     <t>Excel value is unavailable</t>
@@ -870,7 +870,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-14FD-49BF-A292-2B7F6D3ADF81}"/>
+              <c16:uniqueId val="{00000000-0CA8-4ABF-9CF3-B9E4AC90133C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
docs: publish Russian Excel and Word outputs
</commit_message>
<xml_diff>
--- a/1/app/output/ground_truth.xlsx
+++ b/1/app/output/ground_truth.xlsx
@@ -8,31 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Economic analysis of knowledge‑intensive industries\1\app\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF39CD3E-8BC3-44A4-A9F0-6522EE54529B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F6F88E-26FC-4D47-8592-6AB1BC3CA962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3624" yWindow="3624" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Source Data" sheetId="1" r:id="rId1"/>
-    <sheet name="Metrics" sheetId="2" r:id="rId2"/>
-    <sheet name="Costs" sheetId="3" r:id="rId3"/>
+    <sheet name="Исходные данные" sheetId="1" r:id="rId1"/>
+    <sheet name="Метрики" sheetId="2" r:id="rId2"/>
+    <sheet name="Затраты" sheetId="3" r:id="rId3"/>
     <sheet name="TTM" sheetId="4" r:id="rId4"/>
-    <sheet name="Stress Test" sheetId="5" r:id="rId5"/>
-    <sheet name="Harness Log" sheetId="6" r:id="rId6"/>
-    <sheet name="OPEX" sheetId="7" r:id="rId7"/>
-    <sheet name="Assumptions" sheetId="8" r:id="rId8"/>
-    <sheet name="Data Issues" sheetId="9" r:id="rId9"/>
+    <sheet name="Стресс-тест" sheetId="5" r:id="rId5"/>
+    <sheet name="Журнал сверки" sheetId="6" r:id="rId6"/>
+    <sheet name="Структура OPEX" sheetId="7" r:id="rId7"/>
+    <sheet name="Допущения" sheetId="8" r:id="rId8"/>
+    <sheet name="Проблемы данных" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_FilterDatabase" localSheetId="7" hidden="1">Assumptions!$A$1:$F$4</definedName>
-    <definedName name="_FilterDatabase" localSheetId="2" hidden="1">Costs!$A$1:$F$7</definedName>
-    <definedName name="_FilterDatabase" localSheetId="8" hidden="1">'Data Issues'!$A$1:$E$4</definedName>
-    <definedName name="_FilterDatabase" localSheetId="5" hidden="1">'Harness Log'!$A$1:$I$1</definedName>
-    <definedName name="_FilterDatabase" localSheetId="1" hidden="1">Metrics!$A$1:$F$15</definedName>
-    <definedName name="_FilterDatabase" localSheetId="6" hidden="1">OPEX!$A$1:$B$6</definedName>
-    <definedName name="_FilterDatabase" localSheetId="0" hidden="1">'Source Data'!$A$1:$E$37</definedName>
-    <definedName name="_FilterDatabase" localSheetId="4" hidden="1">'Stress Test'!$A$1:$F$8</definedName>
     <definedName name="_FilterDatabase" localSheetId="3" hidden="1">TTM!$A$1:$H$5</definedName>
+    <definedName name="_FilterDatabase" localSheetId="7" hidden="1">Допущения!$A$1:$F$4</definedName>
+    <definedName name="_FilterDatabase" localSheetId="5" hidden="1">'Журнал сверки'!$A$1:$I$1</definedName>
+    <definedName name="_FilterDatabase" localSheetId="2" hidden="1">Затраты!$A$1:$F$7</definedName>
+    <definedName name="_FilterDatabase" localSheetId="0" hidden="1">'Исходные данные'!$A$1:$F$37</definedName>
+    <definedName name="_FilterDatabase" localSheetId="1" hidden="1">Метрики!$A$1:$F$15</definedName>
+    <definedName name="_FilterDatabase" localSheetId="8" hidden="1">'Проблемы данных'!$A$1:$E$4</definedName>
+    <definedName name="_FilterDatabase" localSheetId="4" hidden="1">'Стресс-тест'!$A$1:$F$8</definedName>
+    <definedName name="_FilterDatabase" localSheetId="6" hidden="1">'Структура OPEX'!$A$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
@@ -53,651 +53,696 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="215">
-  <si>
-    <t>Scenario</t>
-  </si>
-  <si>
-    <t>Parameter</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Baseline</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="230">
+  <si>
+    <t>Сценарий</t>
+  </si>
+  <si>
+    <t>Параметр</t>
+  </si>
+  <si>
+    <t>Техническое имя CSV</t>
+  </si>
+  <si>
+    <t>Значение</t>
+  </si>
+  <si>
+    <t>Единица измерения</t>
+  </si>
+  <si>
+    <t>Описание</t>
+  </si>
+  <si>
+    <t>Базовый</t>
+  </si>
+  <si>
+    <t>Календарное время</t>
   </si>
   <si>
     <t>Calendar_Hours</t>
   </si>
   <si>
-    <t>hours</t>
-  </si>
-  <si>
-    <t>Календарный фонд времени в месяц (30 дней * 24 часа)</t>
+    <t>ч</t>
+  </si>
+  <si>
+    <t>Общее календарное время расчётного периода</t>
+  </si>
+  <si>
+    <t>Плановое время работы</t>
   </si>
   <si>
     <t>Planned_Hours</t>
   </si>
   <si>
-    <t>Плановое время работы (2 смены по 8 часов, 30 дней)</t>
+    <t>Запланированное время работы оборудования</t>
+  </si>
+  <si>
+    <t>Фактическое время работы</t>
   </si>
   <si>
     <t>Actual_Hours</t>
   </si>
   <si>
-    <t>Фактическое время реакции (вычет остановок на глубокую промывку и регенерацию)</t>
+    <t>Фактическое время работы оборудования</t>
+  </si>
+  <si>
+    <t>Плановый выпуск</t>
   </si>
   <si>
     <t>Target_Output</t>
   </si>
   <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>Плановый объем выпуска ультрачистого EUV-фоторезиста за плановое время</t>
+    <t>л</t>
+  </si>
+  <si>
+    <t>Плановый объём выпуска</t>
+  </si>
+  <si>
+    <t>Фактический выпуск</t>
   </si>
   <si>
     <t>Actual_Output</t>
   </si>
   <si>
-    <t>Фактически запущенный в синтез объем партии</t>
+    <t>Фактически обработанный объём</t>
+  </si>
+  <si>
+    <t>Годный объём первого прохода</t>
   </si>
   <si>
     <t>First_Pass_Good_Units</t>
   </si>
   <si>
-    <t>Годная продукция с первого прохода без повторной фильтрации (G_fr), FPY = 75%</t>
+    <t>Объём, прошедший контроль с первого раза</t>
+  </si>
+  <si>
+    <t>Итоговый годный объём</t>
   </si>
   <si>
     <t>Final_Good_Units</t>
   </si>
   <si>
-    <t>Итоговая годная продукция после ректификации и переделки (G_final), Final Yield = 85%</t>
+    <t>Итоговый годный объём после переделки</t>
+  </si>
+  <si>
+    <t>Затраты на сырьё</t>
   </si>
   <si>
     <t>Raw_Material_Cost</t>
   </si>
   <si>
-    <t>USD</t>
-  </si>
-  <si>
-    <t>Прямые материалы (DM): прекурсоры олова (SnOx), фотоактивные генераторы, фторированные растворители ($2500/л)</t>
+    <t>долл. США</t>
+  </si>
+  <si>
+    <t>Стоимость использованных сырья и материалов</t>
+  </si>
+  <si>
+    <t>Потребление электроэнергии</t>
   </si>
   <si>
     <t>Energy_kWh</t>
   </si>
   <si>
-    <t>kWh</t>
-  </si>
-  <si>
-    <t>Потребление электроэнергии (криогенный синтез, ISO Class 3 чистые комнаты, глубокий вакуум)</t>
+    <t>кВт·ч</t>
+  </si>
+  <si>
+    <t>Потребление электроэнергии за период</t>
+  </si>
+  <si>
+    <t>Тариф на электроэнергию</t>
   </si>
   <si>
     <t>Energy_Cost_Rate</t>
   </si>
   <si>
-    <t>USD/kWh</t>
-  </si>
-  <si>
-    <t>Тариф на электроэнергию с учетом резервирования мощности</t>
+    <t>долл. США/кВт·ч</t>
+  </si>
+  <si>
+    <t>Стоимость одного киловатт-часа</t>
+  </si>
+  <si>
+    <t>Капитальная стоимость оборудования</t>
   </si>
   <si>
     <t>Equipment_CAPEX</t>
   </si>
   <si>
-    <t>Капитальные затраты: Cleanroom ISO 3, ректорный скид, масс-спектрометры ICP-MS, NMR-спектрометр</t>
+    <t>Первоначальная стоимость оборудования</t>
+  </si>
+  <si>
+    <t>Экономический срок амортизации</t>
   </si>
   <si>
     <t>Amortization_Years_Economic</t>
   </si>
   <si>
-    <t>years</t>
-  </si>
-  <si>
-    <t>Управленческий срок морального износа оборудования (быстрая смена узлов литографии)</t>
+    <t>лет</t>
+  </si>
+  <si>
+    <t>Экономический срок службы оборудования</t>
+  </si>
+  <si>
+    <t>Накладные операционные расходы</t>
   </si>
   <si>
     <t>OPEX_Overhead</t>
   </si>
   <si>
-    <t>USD/month</t>
-  </si>
-  <si>
-    <t>Косвенные расходы: HVAC (вентиляция чистых комнат), азот 99.9999%, утилизация опасных отходов, метрология</t>
+    <t>долл. США/месяц</t>
+  </si>
+  <si>
+    <t>Накладные операционные расходы за период</t>
+  </si>
+  <si>
+    <t>Задержка вывода на рынок</t>
   </si>
   <si>
     <t>Delay_Years</t>
   </si>
   <si>
-    <t>Задержка квалификации фоторезиста у заказчика (Delta t = 6 месяцев)</t>
+    <t>Задержка выхода продукта на рынок</t>
+  </si>
+  <si>
+    <t>Ставка дисконтирования</t>
   </si>
   <si>
     <t>Discount_Rate</t>
   </si>
   <si>
-    <t>ratio</t>
-  </si>
-  <si>
-    <t>Ставка дисконтирования проекта (r = 12% годовых)</t>
+    <t>доля</t>
+  </si>
+  <si>
+    <t>Годовая ставка дисконтирования</t>
+  </si>
+  <si>
+    <t>Темп ценовой эрозии</t>
   </si>
   <si>
     <t>Price_Erosion_Rate</t>
   </si>
   <si>
-    <t>Темп ежегодного падения цены из-за действий конкурентов (alpha = 18% в год)</t>
+    <t>Годовой темп снижения рыночной цены</t>
+  </si>
+  <si>
+    <t>Рыночный горизонт</t>
   </si>
   <si>
     <t>Market_Horizon</t>
   </si>
   <si>
-    <t>Полный жизненный цикл одного состава фоторезиста на рынке (T = 3 года)</t>
+    <t>Доступный горизонт продаж</t>
+  </si>
+  <si>
+    <t>Открытость рыночного окна</t>
   </si>
   <si>
     <t>Market_Window_Open</t>
   </si>
   <si>
-    <t>binary</t>
-  </si>
-  <si>
-    <t>Статус рыночного окна (1 - окно открыто, 0 - заказчик перешел на продукт конкурента)</t>
-  </si>
-  <si>
-    <t>Stress</t>
-  </si>
-  <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t>Volume</t>
-  </si>
-  <si>
-    <t>OPEX</t>
-  </si>
-  <si>
-    <t>CAPEX</t>
-  </si>
-  <si>
-    <t>TTM</t>
-  </si>
-  <si>
-    <t>Metric</t>
-  </si>
-  <si>
-    <t>Formula</t>
-  </si>
-  <si>
-    <t>Parameters</t>
-  </si>
-  <si>
-    <t>Comment</t>
-  </si>
-  <si>
-    <t>FPY</t>
-  </si>
-  <si>
-    <t>G_fr / N</t>
-  </si>
-  <si>
-    <t>First_Pass_Good_Units, Actual_Output</t>
-  </si>
-  <si>
-    <t>dimensionless</t>
-  </si>
-  <si>
-    <t>First-pass yield; not Final Yield</t>
-  </si>
-  <si>
-    <t>Final Yield</t>
-  </si>
-  <si>
-    <t>G_final / N</t>
-  </si>
-  <si>
-    <t>Final_Good_Units, Actual_Output</t>
-  </si>
-  <si>
-    <t>Final good output after rework</t>
-  </si>
-  <si>
-    <t>Availability</t>
-  </si>
-  <si>
-    <t>Actual_Hours / Planned_Hours</t>
-  </si>
-  <si>
-    <t>Actual_Hours, Planned_Hours</t>
-  </si>
-  <si>
-    <t>OEE availability factor</t>
-  </si>
-  <si>
-    <t>Performance</t>
-  </si>
-  <si>
-    <t>(Planned_Hours / Target_Output) * Actual_Output / Actual_Hours</t>
-  </si>
-  <si>
-    <t>Planned_Hours, Target_Output, Actual_Output, Actual_Hours</t>
-  </si>
-  <si>
-    <t>Normative cycle time is derived as h/L</t>
-  </si>
-  <si>
-    <t>Quality</t>
-  </si>
-  <si>
-    <t>Quality = FPY</t>
-  </si>
-  <si>
-    <t>Lecture definition</t>
-  </si>
-  <si>
-    <t>OEE</t>
-  </si>
-  <si>
-    <t>Availability * Performance * Quality</t>
-  </si>
-  <si>
-    <t>Availability, Performance, Quality</t>
-  </si>
-  <si>
-    <t>Operational equipment effectiveness</t>
-  </si>
-  <si>
-    <t>Utilization</t>
-  </si>
-  <si>
-    <t>Planned_Hours / Calendar_Hours</t>
-  </si>
-  <si>
-    <t>Planned_Hours, Calendar_Hours</t>
-  </si>
-  <si>
-    <t>Calendar-time utilization</t>
-  </si>
-  <si>
-    <t>TEEP</t>
-  </si>
-  <si>
-    <t>OEE * Utilization</t>
-  </si>
-  <si>
-    <t>OEE, Utilization</t>
-  </si>
-  <si>
-    <t>CAPEX utilization view</t>
-  </si>
-  <si>
-    <t>Energy Intensity</t>
-  </si>
-  <si>
-    <t>Energy_kWh / Final_Good_Units</t>
-  </si>
-  <si>
-    <t>Energy_kWh, Final_Good_Units</t>
-  </si>
-  <si>
-    <t>kWh/L</t>
-  </si>
-  <si>
-    <t>Gate-to-gate energy use per final good liter</t>
-  </si>
-  <si>
-    <t>Economic Intensity</t>
-  </si>
-  <si>
-    <t>Total Cost / Final Good Units</t>
-  </si>
-  <si>
-    <t>Costs!D4, Final_Good_Units</t>
-  </si>
-  <si>
-    <t>USD/L</t>
-  </si>
-  <si>
-    <t>Numerically equals CPU for this scope</t>
-  </si>
-  <si>
-    <t>CPU</t>
-  </si>
-  <si>
-    <t>Cost per final good liter</t>
-  </si>
-  <si>
-    <t>Mass Intensity</t>
-  </si>
-  <si>
-    <t>Raw material mass / Final Good Units</t>
+    <t>0 или 1</t>
+  </si>
+  <si>
+    <t>Признак открытого рыночного окна</t>
+  </si>
+  <si>
+    <t>Стрессовый</t>
+  </si>
+  <si>
+    <t>Метрика</t>
+  </si>
+  <si>
+    <t>Пояснение формулы</t>
+  </si>
+  <si>
+    <t>Используемые параметры</t>
+  </si>
+  <si>
+    <t>Комментарий</t>
+  </si>
+  <si>
+    <t>Выход годных с первого прохода (FPY)</t>
+  </si>
+  <si>
+    <t>Годный объём первого прохода / фактический выпуск</t>
+  </si>
+  <si>
+    <t>Годный объём первого прохода; фактический выпуск</t>
+  </si>
+  <si>
+    <t>безразмерная величина</t>
+  </si>
+  <si>
+    <t>Доля продукции, прошедшей контроль качества без переделки</t>
+  </si>
+  <si>
+    <t>Итоговый выход годных</t>
+  </si>
+  <si>
+    <t>Итоговый годный объём / фактический выпуск</t>
+  </si>
+  <si>
+    <t>Итоговый годный объём; фактический выпуск</t>
+  </si>
+  <si>
+    <t>Учитывает годную продукцию после переделки</t>
+  </si>
+  <si>
+    <t>Доступность оборудования</t>
+  </si>
+  <si>
+    <t>Фактическое время работы / плановое время работы</t>
+  </si>
+  <si>
+    <t>Фактическое время работы; плановое время работы</t>
+  </si>
+  <si>
+    <t>Коэффициент доступности в составе OEE</t>
+  </si>
+  <si>
+    <t>Производительность оборудования</t>
+  </si>
+  <si>
+    <t>(Плановое время / плановый выпуск) × фактический выпуск / фактическое время</t>
+  </si>
+  <si>
+    <t>Плановое время; плановый выпуск; фактический выпуск; фактическое время</t>
+  </si>
+  <si>
+    <t>Нормативное время цикла рассчитано в часах на литр</t>
+  </si>
+  <si>
+    <t>Коэффициент качества</t>
+  </si>
+  <si>
+    <t>Коэффициент качества = FPY</t>
+  </si>
+  <si>
+    <t>Определение коэффициента качества по лекции</t>
+  </si>
+  <si>
+    <t>Общая эффективность оборудования (OEE)</t>
+  </si>
+  <si>
+    <t>Доступность × производительность × качество</t>
+  </si>
+  <si>
+    <t>Доступность; производительность; качество</t>
+  </si>
+  <si>
+    <t>Операционная эффективность оборудования</t>
+  </si>
+  <si>
+    <t>Использование календарного времени</t>
+  </si>
+  <si>
+    <t>Плановое время работы / календарное время</t>
+  </si>
+  <si>
+    <t>Плановое время работы; календарное время</t>
+  </si>
+  <si>
+    <t>Использование доступного календарного фонда времени</t>
+  </si>
+  <si>
+    <t>Полная эффективная производительность оборудования (TEEP)</t>
+  </si>
+  <si>
+    <t>OEE × использование календарного времени</t>
+  </si>
+  <si>
+    <t>OEE; использование календарного времени</t>
+  </si>
+  <si>
+    <t>Показывает использование производственного потенциала CAPEX</t>
+  </si>
+  <si>
+    <t>Энергетическая ресурсоёмкость</t>
+  </si>
+  <si>
+    <t>Потребление электроэнергии / итоговый годный объём</t>
+  </si>
+  <si>
+    <t>Потребление электроэнергии; итоговый годный объём</t>
+  </si>
+  <si>
+    <t>кВт·ч/л</t>
+  </si>
+  <si>
+    <t>Потребление энергии на литр итоговой годной продукции</t>
+  </si>
+  <si>
+    <t>Экономическая ресурсоёмкость</t>
+  </si>
+  <si>
+    <t>Общие производственные затраты / итоговый годный объём</t>
+  </si>
+  <si>
+    <t>Общие производственные затраты; итоговый годный объём</t>
+  </si>
+  <si>
+    <t>долл. США/л</t>
+  </si>
+  <si>
+    <t>В данной области расчёта численно совпадает с CPU</t>
+  </si>
+  <si>
+    <t>Себестоимость единицы продукции (CPU)</t>
+  </si>
+  <si>
+    <t>Себестоимость литра итоговой годной продукции</t>
+  </si>
+  <si>
+    <t>Массовая ресурсоёмкость</t>
+  </si>
+  <si>
+    <t>Масса сырья / итоговый годный объём</t>
+  </si>
+  <si>
+    <t>Raw_Material_Mass_kg (масса сырья)</t>
+  </si>
+  <si>
+    <t>НЕ РАССЧИТЫВАЕТСЯ</t>
+  </si>
+  <si>
+    <t>кг/л</t>
+  </si>
+  <si>
+    <t>Параметр Raw_Material_Mass_kg отсутствует в исходных данных</t>
+  </si>
+  <si>
+    <t>Штраф TTM по параметрам задания</t>
+  </si>
+  <si>
+    <t>Мультипликативная потеря сохраняемой стоимости из-за задержки</t>
+  </si>
+  <si>
+    <t>Параметры TTM в строке 2</t>
+  </si>
+  <si>
+    <t>Ставка дисконтирования 10 %, ценовая эрозия 15 %, горизонт 3 года</t>
+  </si>
+  <si>
+    <t>Штраф TTM по параметрам CSV</t>
+  </si>
+  <si>
+    <t>Параметры TTM в строке 3</t>
+  </si>
+  <si>
+    <t>Ставки из CSV показаны отдельным сценарием</t>
+  </si>
+  <si>
+    <t>Затраты на электроэнергию</t>
+  </si>
+  <si>
+    <t>Потребление электроэнергии × тариф</t>
+  </si>
+  <si>
+    <t>Потребление электроэнергии; тариф на электроэнергию</t>
+  </si>
+  <si>
+    <t>Затраты на покупную электроэнергию</t>
+  </si>
+  <si>
+    <t>Ежемесячная амортизация</t>
+  </si>
+  <si>
+    <t>CAPEX / экономический срок / 12</t>
+  </si>
+  <si>
+    <t>Капитальная стоимость; экономический срок амортизации</t>
+  </si>
+  <si>
+    <t>Набор данных за 30 суток принят за один месяц</t>
+  </si>
+  <si>
+    <t>Общие производственные затраты</t>
+  </si>
+  <si>
+    <t>Сырьё + энергия + накладные расходы + амортизация</t>
+  </si>
+  <si>
+    <t>Исходные данные; затраты на электроэнергию; амортизация</t>
+  </si>
+  <si>
+    <t>Прозрачная структура полной производственной стоимости</t>
+  </si>
+  <si>
+    <t>Полная экономическая ресурсоёмкость</t>
+  </si>
+  <si>
+    <t>Себестоимость единицы продукции</t>
+  </si>
+  <si>
+    <t>Стоимостной показатель сырья</t>
+  </si>
+  <si>
+    <t>Затраты на сырьё / итоговый годный объём</t>
+  </si>
+  <si>
+    <t>Затраты на сырьё; итоговый годный объём</t>
+  </si>
+  <si>
+    <t>Стоимостной показатель не заменяет массовую ресурсоёмкость</t>
+  </si>
+  <si>
+    <t>Ценовая эрозия</t>
+  </si>
+  <si>
+    <t>Рыночный горизонт, лет</t>
+  </si>
+  <si>
+    <t>Задержка, лет</t>
+  </si>
+  <si>
+    <t>Рыночное окно открыто</t>
+  </si>
+  <si>
+    <t>Штраф TTM</t>
+  </si>
+  <si>
+    <t>Параметры задания</t>
+  </si>
+  <si>
+    <t>Параметры практического задания</t>
+  </si>
+  <si>
+    <t>Параметры CSV</t>
+  </si>
+  <si>
+    <t>Параметры из исходного CSV</t>
+  </si>
+  <si>
+    <t>Базовый для стресс-теста</t>
+  </si>
+  <si>
+    <t>Задержка из базового столбца сравнительного CSV</t>
+  </si>
+  <si>
+    <t>Задержка из стрессового CSV</t>
+  </si>
+  <si>
+    <t>Базовый сценарий</t>
+  </si>
+  <si>
+    <t>Стрессовый сценарий</t>
+  </si>
+  <si>
+    <t>Абсолютное изменение</t>
+  </si>
+  <si>
+    <t>Относительное изменение</t>
+  </si>
+  <si>
+    <t>Интерпретация</t>
+  </si>
+  <si>
+    <t>Снижается доля годной продукции первого прохода</t>
+  </si>
+  <si>
+    <t>Снижение качества уменьшает общую эффективность оборудования</t>
+  </si>
+  <si>
+    <t>Использование календарного времени не изменяется</t>
+  </si>
+  <si>
+    <t>Трёхкратный тариф увеличивает затраты на электроэнергию</t>
+  </si>
+  <si>
+    <t>Рост затрат повышает стоимость ресурсов на литр годной продукции</t>
+  </si>
+  <si>
+    <t>Численно совпадает с экономической ресурсоёмкостью в текущей области расчёта</t>
+  </si>
+  <si>
+    <t>Штраф за задержку вывода на рынок (TTM)</t>
+  </si>
+  <si>
+    <t>Задержка создаёт мультипликативный экономический штраф</t>
+  </si>
+  <si>
+    <t>Значение Excel</t>
+  </si>
+  <si>
+    <t>Значение Python</t>
+  </si>
+  <si>
+    <t>Абсолютное отклонение</t>
+  </si>
+  <si>
+    <t>Относительное отклонение</t>
+  </si>
+  <si>
+    <t>Допуск</t>
+  </si>
+  <si>
+    <t>Статус</t>
+  </si>
+  <si>
+    <t>Вероятная причина</t>
+  </si>
+  <si>
+    <t>Временная метка</t>
+  </si>
+  <si>
+    <t>СОВПАДАЕТ</t>
+  </si>
+  <si>
+    <t>2026-09-14T08:59:36.107726+00:00</t>
+  </si>
+  <si>
+    <t>Значение Excel недоступно</t>
+  </si>
+  <si>
+    <t>Категория затрат</t>
+  </si>
+  <si>
+    <t>Доля</t>
+  </si>
+  <si>
+    <t>Сырье и прекурсоры</t>
+  </si>
+  <si>
+    <t>Утилиты</t>
+  </si>
+  <si>
+    <t>Персонал</t>
+  </si>
+  <si>
+    <t>ТОиР</t>
+  </si>
+  <si>
+    <t>Комплаенс, качество и метрология</t>
+  </si>
+  <si>
+    <t>Код</t>
+  </si>
+  <si>
+    <t>Допущение</t>
+  </si>
+  <si>
+    <t>Обоснование</t>
+  </si>
+  <si>
+    <t>Влияние</t>
+  </si>
+  <si>
+    <t>Источник</t>
+  </si>
+  <si>
+    <t>A01</t>
+  </si>
+  <si>
+    <t>Расчётный период — один месяц</t>
+  </si>
+  <si>
+    <t>Calendar_Hours = 720 = 30 × 24</t>
+  </si>
+  <si>
+    <t>Месячная амортизация</t>
+  </si>
+  <si>
+    <t>CSV</t>
+  </si>
+  <si>
+    <t>Принято</t>
+  </si>
+  <si>
+    <t>A02</t>
+  </si>
+  <si>
+    <t>Нормативное время цикла = плановое время / плановый выпуск</t>
+  </si>
+  <si>
+    <t>Отдельное поле отсутствует</t>
+  </si>
+  <si>
+    <t>Производительность и OEE</t>
+  </si>
+  <si>
+    <t>Лекция + CSV</t>
+  </si>
+  <si>
+    <t>A03</t>
+  </si>
+  <si>
+    <t>Знаменатель CPU — итоговый годный объём</t>
+  </si>
+  <si>
+    <t>Это объём после итогового контроля</t>
+  </si>
+  <si>
+    <t>CPU и ресурсоёмкость</t>
+  </si>
+  <si>
+    <t>Лекция + задание</t>
+  </si>
+  <si>
+    <t>Проблема</t>
+  </si>
+  <si>
+    <t>Критичность</t>
+  </si>
+  <si>
+    <t>Рекомендуемое действие</t>
+  </si>
+  <si>
+    <t>Отсутствует масса сырья</t>
   </si>
   <si>
     <t>Raw_Material_Mass_kg</t>
   </si>
   <si>
-    <t>NOT_COMPUTABLE</t>
-  </si>
-  <si>
-    <t>kg/L</t>
-  </si>
-  <si>
-    <t>Raw_Material_Mass_kg is absent from source data</t>
-  </si>
-  <si>
-    <t>TTM Penalty Assignment</t>
-  </si>
-  <si>
-    <t>Multiplicative retained-value loss</t>
-  </si>
-  <si>
-    <t>TTM!B2:F2</t>
-  </si>
-  <si>
-    <t>r=10%, alpha=15%, T=3</t>
-  </si>
-  <si>
-    <t>TTM Penalty CSV</t>
-  </si>
-  <si>
-    <t>TTM!B3:F3</t>
-  </si>
-  <si>
-    <t>CSV rates retained separately</t>
-  </si>
-  <si>
-    <t>Energy Cost</t>
-  </si>
-  <si>
-    <t>Energy_kWh * Energy_Cost_Rate</t>
-  </si>
-  <si>
-    <t>Energy_kWh, Energy_Cost_Rate</t>
-  </si>
-  <si>
-    <t>Purchased electricity</t>
-  </si>
-  <si>
-    <t>Monthly Depreciation</t>
-  </si>
-  <si>
-    <t>CAPEX / Economic Life / 12</t>
-  </si>
-  <si>
-    <t>Equipment_CAPEX, Amortization_Years_Economic</t>
-  </si>
-  <si>
-    <t>30-day dataset is treated as one month</t>
-  </si>
-  <si>
-    <t>Total Manufacturing Cost</t>
-  </si>
-  <si>
-    <t>Raw materials + Energy + Overhead + Depreciation</t>
-  </si>
-  <si>
-    <t>Source Data, D2, D3</t>
-  </si>
-  <si>
-    <t>Transparent cost build-up</t>
-  </si>
-  <si>
-    <t>D4, Final_Good_Units</t>
-  </si>
-  <si>
-    <t>Full economic resource intensity</t>
-  </si>
-  <si>
-    <t>Cost per unit</t>
-  </si>
-  <si>
-    <t>Raw Material Cost Proxy</t>
-  </si>
-  <si>
-    <t>Raw Material Cost / Final Good Units</t>
-  </si>
-  <si>
-    <t>Raw_Material_Cost, Final_Good_Units</t>
-  </si>
-  <si>
-    <t>Cost proxy; not mass intensity</t>
-  </si>
-  <si>
-    <t>Discount Rate</t>
-  </si>
-  <si>
-    <t>Price Erosion</t>
-  </si>
-  <si>
-    <t>Market Horizon</t>
-  </si>
-  <si>
-    <t>Delay</t>
-  </si>
-  <si>
-    <t>Window Open</t>
-  </si>
-  <si>
-    <t>Penalty</t>
-  </si>
-  <si>
-    <t>Assignment</t>
-  </si>
-  <si>
-    <t>Task parameters</t>
-  </si>
-  <si>
-    <t>CSV</t>
-  </si>
-  <si>
-    <t>CSV parameters</t>
-  </si>
-  <si>
-    <t>Stress Baseline</t>
-  </si>
-  <si>
-    <t>Delay from comparison CSV baseline</t>
-  </si>
-  <si>
-    <t>Delay from stress CSV</t>
-  </si>
-  <si>
-    <t>Absolute Change</t>
-  </si>
-  <si>
-    <t>Relative Change</t>
-  </si>
-  <si>
-    <t>Interpretation</t>
-  </si>
-  <si>
-    <t>First-pass quality falls</t>
-  </si>
-  <si>
-    <t>Quality reduces equipment effectiveness</t>
-  </si>
-  <si>
-    <t>Calendar utilization is unchanged</t>
-  </si>
-  <si>
-    <t>Threefold tariff raises energy cost</t>
-  </si>
-  <si>
-    <t>Higher energy cost raises cost per good liter</t>
-  </si>
-  <si>
-    <t>Same scoped numerator and denominator as economic intensity</t>
-  </si>
-  <si>
-    <t>TTM Penalty</t>
-  </si>
-  <si>
-    <t>Delay creates a multiplicative economic penalty</t>
-  </si>
-  <si>
-    <t>Excel Value</t>
-  </si>
-  <si>
-    <t>Python Value</t>
-  </si>
-  <si>
-    <t>Absolute Delta</t>
-  </si>
-  <si>
-    <t>Relative Delta</t>
-  </si>
-  <si>
-    <t>Tolerance</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Probable Cause</t>
-  </si>
-  <si>
-    <t>Timestamp</t>
-  </si>
-  <si>
-    <t>PASS</t>
-  </si>
-  <si>
-    <t>2026-09-14T08:16:12.931028+00:00</t>
-  </si>
-  <si>
-    <t>Excel value is unavailable</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Share</t>
-  </si>
-  <si>
-    <t>Сырье и прекурсоры</t>
-  </si>
-  <si>
-    <t>Утилиты</t>
-  </si>
-  <si>
-    <t>Персонал</t>
-  </si>
-  <si>
-    <t>ТОиР</t>
-  </si>
-  <si>
-    <t>Compliance / качество / метрология</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Assumption</t>
-  </si>
-  <si>
-    <t>Reason</t>
-  </si>
-  <si>
-    <t>Impact</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>A01</t>
-  </si>
-  <si>
-    <t>Расчётный период — один месяц</t>
-  </si>
-  <si>
-    <t>Calendar_Hours = 720 = 30 × 24</t>
-  </si>
-  <si>
-    <t>Месячная амортизация</t>
-  </si>
-  <si>
-    <t>Принято</t>
-  </si>
-  <si>
-    <t>A02</t>
-  </si>
-  <si>
-    <t>Normative Cycle Time = Planned_Hours / Target_Output</t>
-  </si>
-  <si>
-    <t>Отдельное поле отсутствует</t>
-  </si>
-  <si>
-    <t>Performance и OEE</t>
-  </si>
-  <si>
-    <t>Лекция + CSV</t>
-  </si>
-  <si>
-    <t>A03</t>
-  </si>
-  <si>
-    <t>Знаменатель CPU — Final_Good_Units</t>
-  </si>
-  <si>
-    <t>Это объём после итогового контроля</t>
-  </si>
-  <si>
-    <t>CPU и intensity</t>
-  </si>
-  <si>
-    <t>Лекция + задание</t>
-  </si>
-  <si>
-    <t>Issue</t>
-  </si>
-  <si>
-    <t>Severity</t>
-  </si>
-  <si>
-    <t>Effect</t>
-  </si>
-  <si>
-    <t>Action</t>
-  </si>
-  <si>
-    <t>Mass input is absent</t>
-  </si>
-  <si>
-    <t>HIGH</t>
-  </si>
-  <si>
-    <t>Mass intensity is NOT_COMPUTABLE</t>
-  </si>
-  <si>
-    <t>Add consumed raw-material mass in kg</t>
-  </si>
-  <si>
-    <t>TTM rates conflict</t>
+    <t>ВЫСОКАЯ</t>
+  </si>
+  <si>
+    <t>Массовая ресурсоёмкость не рассчитывается</t>
+  </si>
+  <si>
+    <t>Добавить массу потреблённого сырья в килограммах</t>
+  </si>
+  <si>
+    <t>Параметры TTM расходятся</t>
   </si>
   <si>
     <t>Discount_Rate; Price_Erosion_Rate</t>
   </si>
   <si>
-    <t>MEDIUM</t>
-  </si>
-  <si>
-    <t>Different TTM penalties</t>
-  </si>
-  <si>
-    <t>Report assignment and CSV scenarios separately</t>
-  </si>
-  <si>
-    <t>Pilot delay differs from comparison baseline</t>
-  </si>
-  <si>
-    <t>Pilot is not the no-delay baseline</t>
-  </si>
-  <si>
-    <t>Use comparison CSV for stress baseline validation</t>
+    <t>СРЕДНЯЯ</t>
+  </si>
+  <si>
+    <t>Получаются разные штрафы TTM</t>
+  </si>
+  <si>
+    <t>Показывать сценарии задания и CSV отдельно</t>
+  </si>
+  <si>
+    <t>Задержка пилотного сценария отличается от базового comparison CSV</t>
+  </si>
+  <si>
+    <t>Пилотный сценарий не является сценарием без задержки</t>
+  </si>
+  <si>
+    <t>Использовать comparison CSV для проверки стресс-сценария</t>
   </si>
 </sst>
 </file>
@@ -787,7 +832,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Структура OPEX в High-Tech производстве</a:t>
+              <a:t>Структура OPEX в высокотехнологичном производстве</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -806,11 +851,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>OPEX!$B$1</c:f>
+              <c:f>'Структура OPEX'!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Share</c:v>
+                  <c:v>Доля</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -823,7 +868,7 @@
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:strRef>
-              <c:f>OPEX!$A$2:$A$6</c:f>
+              <c:f>'Структура OPEX'!$A$2:$A$6</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -839,14 +884,14 @@
                   <c:v>ТОиР</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Compliance / качество / метрология</c:v>
+                  <c:v>Комплаенс, качество и метрология</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>OPEX!$B$2:$B$6</c:f>
+              <c:f>'Структура OPEX'!$B$2:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -870,7 +915,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-0CA8-4ABF-9CF3-B9E4AC90133C}"/>
+              <c16:uniqueId val="{00000000-E6C5-4274-8E61-F763DFF8B5D4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1328,17 +1373,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="72" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1354,621 +1400,732 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2">
+        <v>720</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="C2">
-        <v>720</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
       <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3">
+        <v>480</v>
+      </c>
+      <c r="E3" t="s">
         <v>9</v>
       </c>
-      <c r="C3">
-        <v>480</v>
-      </c>
-      <c r="D3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4">
         <v>390</v>
       </c>
-      <c r="D4" t="s">
-        <v>7</v>
-      </c>
       <c r="E4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5">
         <v>120</v>
       </c>
-      <c r="D5" t="s">
-        <v>14</v>
-      </c>
       <c r="E5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6">
         <v>95</v>
       </c>
-      <c r="D6" t="s">
-        <v>14</v>
-      </c>
       <c r="E6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7">
         <v>71.25</v>
-      </c>
-      <c r="D7" t="s">
-        <v>14</v>
       </c>
       <c r="E7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8">
         <v>80.75</v>
       </c>
-      <c r="D8" t="s">
-        <v>14</v>
-      </c>
       <c r="E8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9">
         <v>240000</v>
       </c>
-      <c r="D9" t="s">
-        <v>23</v>
-      </c>
       <c r="E9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10">
         <v>115000</v>
       </c>
-      <c r="D10" t="s">
-        <v>26</v>
-      </c>
       <c r="E10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+      <c r="F10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11">
         <v>0.22</v>
       </c>
-      <c r="D11" t="s">
-        <v>29</v>
-      </c>
       <c r="E11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="F11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12">
+        <v>42</v>
+      </c>
+      <c r="C12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12">
         <v>28000000</v>
-      </c>
-      <c r="D12" t="s">
-        <v>23</v>
       </c>
       <c r="E12" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13">
         <v>3</v>
       </c>
-      <c r="D13" t="s">
-        <v>34</v>
-      </c>
       <c r="E13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="F13" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14">
+        <v>49</v>
+      </c>
+      <c r="C14" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14">
         <v>145000</v>
       </c>
-      <c r="D14" t="s">
-        <v>37</v>
-      </c>
       <c r="E14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+      <c r="F14" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15">
+        <v>53</v>
+      </c>
+      <c r="C15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15">
         <v>0.5</v>
       </c>
-      <c r="D15" t="s">
-        <v>34</v>
-      </c>
       <c r="E15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="F15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16">
+        <v>56</v>
+      </c>
+      <c r="C16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16">
         <v>0.12</v>
       </c>
-      <c r="D16" t="s">
-        <v>42</v>
-      </c>
       <c r="E16" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+      <c r="F16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17">
+        <v>60</v>
+      </c>
+      <c r="C17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17">
         <v>0.18</v>
       </c>
-      <c r="D17" t="s">
-        <v>42</v>
-      </c>
       <c r="E17" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+      <c r="F17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18">
+        <v>63</v>
+      </c>
+      <c r="C18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18">
         <v>3</v>
-      </c>
-      <c r="D18" t="s">
-        <v>34</v>
       </c>
       <c r="E18" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B19" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20">
+        <v>720</v>
+      </c>
+      <c r="E20" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21">
+        <v>480</v>
+      </c>
+      <c r="E21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22">
+        <v>390</v>
+      </c>
+      <c r="E22" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23">
+        <v>120</v>
+      </c>
+      <c r="E23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24">
+        <v>95</v>
+      </c>
+      <c r="E24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25">
+        <v>38</v>
+      </c>
+      <c r="E25" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26">
+        <v>80.75</v>
+      </c>
+      <c r="E26" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>70</v>
+      </c>
+      <c r="B27" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" t="s">
+        <v>31</v>
+      </c>
+      <c r="D27">
+        <v>240000</v>
+      </c>
+      <c r="E27" t="s">
+        <v>32</v>
+      </c>
+      <c r="F27" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>70</v>
+      </c>
+      <c r="B28" t="s">
+        <v>34</v>
+      </c>
+      <c r="C28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28">
+        <v>115000</v>
+      </c>
+      <c r="E28" t="s">
+        <v>36</v>
+      </c>
+      <c r="F28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>70</v>
+      </c>
+      <c r="B29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29">
+        <v>0.66</v>
+      </c>
+      <c r="E29" t="s">
+        <v>40</v>
+      </c>
+      <c r="F29" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" t="s">
+        <v>43</v>
+      </c>
+      <c r="D30">
+        <v>28000000</v>
+      </c>
+      <c r="E30" t="s">
+        <v>32</v>
+      </c>
+      <c r="F30" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" t="s">
+        <v>45</v>
+      </c>
+      <c r="C31" t="s">
+        <v>46</v>
+      </c>
+      <c r="D31">
+        <v>3</v>
+      </c>
+      <c r="E31" t="s">
+        <v>47</v>
+      </c>
+      <c r="F31" t="s">
         <v>48</v>
       </c>
-      <c r="C19">
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>70</v>
+      </c>
+      <c r="B32" t="s">
+        <v>49</v>
+      </c>
+      <c r="C32" t="s">
+        <v>50</v>
+      </c>
+      <c r="D32">
+        <v>145000</v>
+      </c>
+      <c r="E32" t="s">
+        <v>51</v>
+      </c>
+      <c r="F32" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" t="s">
+        <v>54</v>
+      </c>
+      <c r="D33">
+        <v>0.5</v>
+      </c>
+      <c r="E33" t="s">
+        <v>47</v>
+      </c>
+      <c r="F33" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B34" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34">
+        <v>0.12</v>
+      </c>
+      <c r="E34" t="s">
+        <v>58</v>
+      </c>
+      <c r="F34" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>70</v>
+      </c>
+      <c r="B35" t="s">
+        <v>60</v>
+      </c>
+      <c r="C35" t="s">
+        <v>61</v>
+      </c>
+      <c r="D35">
+        <v>0.18</v>
+      </c>
+      <c r="E35" t="s">
+        <v>58</v>
+      </c>
+      <c r="F35" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36" t="s">
+        <v>64</v>
+      </c>
+      <c r="D36">
+        <v>3</v>
+      </c>
+      <c r="E36" t="s">
+        <v>47</v>
+      </c>
+      <c r="F36" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>70</v>
+      </c>
+      <c r="B37" t="s">
+        <v>66</v>
+      </c>
+      <c r="C37" t="s">
+        <v>67</v>
+      </c>
+      <c r="D37">
         <v>1</v>
       </c>
-      <c r="D19" t="s">
-        <v>49</v>
-      </c>
-      <c r="E19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>51</v>
-      </c>
-      <c r="B20" t="s">
-        <v>6</v>
-      </c>
-      <c r="C20">
-        <v>720</v>
-      </c>
-      <c r="D20" t="s">
-        <v>7</v>
-      </c>
-      <c r="E20" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>51</v>
-      </c>
-      <c r="B21" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21">
-        <v>480</v>
-      </c>
-      <c r="D21" t="s">
-        <v>7</v>
-      </c>
-      <c r="E21" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22">
-        <v>390</v>
-      </c>
-      <c r="D22" t="s">
-        <v>7</v>
-      </c>
-      <c r="E22" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23">
-        <v>120</v>
-      </c>
-      <c r="D23" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>51</v>
-      </c>
-      <c r="B24" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24">
-        <v>95</v>
-      </c>
-      <c r="D24" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>51</v>
-      </c>
-      <c r="B25" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25">
-        <v>38</v>
-      </c>
-      <c r="D25" t="s">
-        <v>14</v>
-      </c>
-      <c r="E25" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>51</v>
-      </c>
-      <c r="B26" t="s">
-        <v>20</v>
-      </c>
-      <c r="C26">
-        <v>80.75</v>
-      </c>
-      <c r="D26" t="s">
-        <v>14</v>
-      </c>
-      <c r="E26" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>51</v>
-      </c>
-      <c r="B27" t="s">
-        <v>22</v>
-      </c>
-      <c r="C27">
-        <v>240000</v>
-      </c>
-      <c r="D27" t="s">
-        <v>23</v>
-      </c>
-      <c r="E27" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>51</v>
-      </c>
-      <c r="B28" t="s">
-        <v>25</v>
-      </c>
-      <c r="C28">
-        <v>115000</v>
-      </c>
-      <c r="D28" t="s">
-        <v>26</v>
-      </c>
-      <c r="E28" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>51</v>
-      </c>
-      <c r="B29" t="s">
-        <v>28</v>
-      </c>
-      <c r="C29">
-        <v>0.66</v>
-      </c>
-      <c r="D29" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>51</v>
-      </c>
-      <c r="B30" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30">
-        <v>28000000</v>
-      </c>
-      <c r="D30" t="s">
-        <v>23</v>
-      </c>
-      <c r="E30" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>51</v>
-      </c>
-      <c r="B31" t="s">
-        <v>33</v>
-      </c>
-      <c r="C31">
-        <v>3</v>
-      </c>
-      <c r="D31" t="s">
-        <v>34</v>
-      </c>
-      <c r="E31" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>51</v>
-      </c>
-      <c r="B32" t="s">
-        <v>36</v>
-      </c>
-      <c r="C32">
-        <v>145000</v>
-      </c>
-      <c r="D32" t="s">
-        <v>37</v>
-      </c>
-      <c r="E32" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>51</v>
-      </c>
-      <c r="B33" t="s">
-        <v>39</v>
-      </c>
-      <c r="C33">
-        <v>0.5</v>
-      </c>
-      <c r="D33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E33" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>51</v>
-      </c>
-      <c r="B34" t="s">
-        <v>41</v>
-      </c>
-      <c r="C34">
-        <v>0.12</v>
-      </c>
-      <c r="D34" t="s">
-        <v>42</v>
-      </c>
-      <c r="E34" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>51</v>
-      </c>
-      <c r="B35" t="s">
-        <v>44</v>
-      </c>
-      <c r="C35">
-        <v>0.18</v>
-      </c>
-      <c r="D35" t="s">
-        <v>42</v>
-      </c>
-      <c r="E35" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>51</v>
-      </c>
-      <c r="B36" t="s">
-        <v>46</v>
-      </c>
-      <c r="C36">
-        <v>3</v>
-      </c>
-      <c r="D36" t="s">
-        <v>34</v>
-      </c>
-      <c r="E36" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>51</v>
-      </c>
-      <c r="B37" t="s">
-        <v>48</v>
-      </c>
-      <c r="C37">
-        <v>1</v>
-      </c>
-      <c r="D37" t="s">
-        <v>49</v>
-      </c>
       <c r="E37" t="s">
-        <v>56</v>
+        <v>68</v>
+      </c>
+      <c r="F37" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E37" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F37" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1988,315 +2145,315 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D2">
-        <f>'Source Data'!$C$7/'Source Data'!$C$6</f>
+        <v>77</v>
+      </c>
+      <c r="D2" s="2">
+        <f>'Исходные данные'!$D$7/'Исходные данные'!$D$6</f>
         <v>0.75</v>
       </c>
       <c r="E2" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D3">
-        <f>'Source Data'!$C$8/'Source Data'!$C$6</f>
+        <v>82</v>
+      </c>
+      <c r="D3" s="2">
+        <f>'Исходные данные'!$D$8/'Исходные данные'!$D$6</f>
         <v>0.85</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D4">
-        <f>'Source Data'!$C$4/'Source Data'!$C$3</f>
+        <v>86</v>
+      </c>
+      <c r="D4" s="2">
+        <f>'Исходные данные'!$D$4/'Исходные данные'!$D$3</f>
         <v>0.8125</v>
       </c>
       <c r="E4" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D5">
-        <f>('Source Data'!$C$3/'Source Data'!$C$5)*'Source Data'!$C$6/'Source Data'!$C$4</f>
+        <v>90</v>
+      </c>
+      <c r="D5" s="2">
+        <f>('Исходные данные'!$D$3/'Исходные данные'!$D$5)*'Исходные данные'!$D$6/'Исходные данные'!$D$4</f>
         <v>0.97435897435897434</v>
       </c>
       <c r="E5" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D6">
+        <v>75</v>
+      </c>
+      <c r="D6" s="2">
         <f>D2</f>
         <v>0.75</v>
       </c>
       <c r="E6" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7">
+        <v>97</v>
+      </c>
+      <c r="D7" s="2">
         <f>D4*D5*D6</f>
         <v>0.59375</v>
       </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="C8" t="s">
-        <v>87</v>
-      </c>
-      <c r="D8">
-        <f>'Source Data'!$C$3/'Source Data'!$C$2</f>
+        <v>101</v>
+      </c>
+      <c r="D8" s="2">
+        <f>'Исходные данные'!$D$3/'Исходные данные'!$D$2</f>
         <v>0.66666666666666663</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F8" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="B9" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D9">
+        <v>105</v>
+      </c>
+      <c r="D9" s="2">
         <f>D7*D8</f>
         <v>0.39583333333333331</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F9" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="B10" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C10" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="D10">
-        <f>'Source Data'!$C$10/'Source Data'!$C$8</f>
+        <f>'Исходные данные'!$D$10/'Исходные данные'!$D$8</f>
         <v>1424.1486068111456</v>
       </c>
       <c r="E10" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="F10" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="B11" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="D11">
-        <f>Costs!D5</f>
+        <f>Затраты!D5</f>
         <v>14713.037495700037</v>
       </c>
       <c r="E11" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="F11" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B12" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="C12" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="D12">
-        <f>Costs!D6</f>
+        <f>Затраты!D6</f>
         <v>14713.037495700037</v>
       </c>
       <c r="E12" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="F12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B13" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="C13" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="D13" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="E13" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="F13" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C14" t="s">
-        <v>113</v>
-      </c>
-      <c r="D14">
+        <v>127</v>
+      </c>
+      <c r="D14" s="2">
         <f>TTM!G2</f>
         <v>0.26285941114120437</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F14" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B15" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C15" t="s">
-        <v>116</v>
-      </c>
-      <c r="D15">
+        <v>130</v>
+      </c>
+      <c r="D15" s="2">
         <f>TTM!G3</f>
         <v>0.2803468358172122</v>
       </c>
       <c r="E15" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F15" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2320,148 +2477,148 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B2" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C2" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="D2">
-        <f>'Source Data'!$C$10*'Source Data'!$C$11</f>
+        <f>'Исходные данные'!$D$10*'Исходные данные'!$D$11</f>
         <v>25300</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="B3" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="C3" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="D3">
-        <f>'Source Data'!$C$12/'Source Data'!$C$13/12</f>
+        <f>'Исходные данные'!$D$12/'Исходные данные'!$D$13/12</f>
         <v>777777.77777777787</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="B4" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="C4" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="D4">
-        <f>'Source Data'!$C$9+D2+'Source Data'!$C$14+D3</f>
+        <f>'Исходные данные'!$D$9+D2+'Исходные данные'!$D$14+D3</f>
         <v>1188077.777777778</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="C5" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="D5">
-        <f>D4/'Source Data'!$C$8</f>
+        <f>D4/'Исходные данные'!$D$8</f>
         <v>14713.037495700037</v>
       </c>
       <c r="E5" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="F5" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="C6" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="D6">
-        <f>D4/'Source Data'!$C$8</f>
+        <f>D4/'Исходные данные'!$D$8</f>
         <v>14713.037495700037</v>
       </c>
       <c r="E6" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="F6" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="C7" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="D7">
-        <f>'Source Data'!$C$9/'Source Data'!$C$8</f>
+        <f>'Исходные данные'!$D$9/'Исходные данные'!$D$8</f>
         <v>2972.1362229102169</v>
       </c>
       <c r="E7" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="F7" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -2487,30 +2644,30 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>137</v>
+        <v>56</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="B2" s="2">
         <v>0.1</v>
@@ -2532,12 +2689,12 @@
         <v>0.26285941114120437</v>
       </c>
       <c r="H2" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B3" s="2">
         <v>0.12</v>
@@ -2559,12 +2716,12 @@
         <v>0.2803468358172122</v>
       </c>
       <c r="H3" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="B4" s="2">
         <v>0.1</v>
@@ -2586,12 +2743,12 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="B5" s="2">
         <v>0.1</v>
@@ -2613,7 +2770,7 @@
         <v>0.26285941114120437</v>
       </c>
       <c r="H5" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -2634,34 +2791,34 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>162</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="B2">
-        <f>'Source Data'!$C$7/'Source Data'!$C$6</f>
+        <f>'Исходные данные'!$D$7/'Исходные данные'!$D$6</f>
         <v>0.75</v>
       </c>
       <c r="C2">
-        <f>'Source Data'!$C$25/'Source Data'!$C$24</f>
+        <f>'Исходные данные'!$D$25/'Исходные данные'!$D$24</f>
         <v>0.4</v>
       </c>
       <c r="D2">
@@ -2673,19 +2830,19 @@
         <v>-0.46666666666666662</v>
       </c>
       <c r="F2" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="B3">
-        <f>('Source Data'!$C$4/'Source Data'!$C$3)*(('Source Data'!$C$3/'Source Data'!$C$5)*'Source Data'!$C$6/'Source Data'!$C$4)*('Source Data'!$C$7/'Source Data'!$C$6)</f>
+        <f>('Исходные данные'!$D$4/'Исходные данные'!$D$3)*(('Исходные данные'!$D$3/'Исходные данные'!$D$5)*'Исходные данные'!$D$6/'Исходные данные'!$D$4)*('Исходные данные'!$D$7/'Исходные данные'!$D$6)</f>
         <v>0.59375</v>
       </c>
       <c r="C3">
-        <f>('Source Data'!$C$22/'Source Data'!$C$21)*(('Source Data'!$C$21/'Source Data'!$C$23)*'Source Data'!$C$24/'Source Data'!$C$22)*('Source Data'!$C$25/'Source Data'!$C$24)</f>
+        <f>('Исходные данные'!$D$22/'Исходные данные'!$D$21)*(('Исходные данные'!$D$21/'Исходные данные'!$D$23)*'Исходные данные'!$D$24/'Исходные данные'!$D$22)*('Исходные данные'!$D$25/'Исходные данные'!$D$24)</f>
         <v>0.31666666666666665</v>
       </c>
       <c r="D3">
@@ -2697,19 +2854,19 @@
         <v>-0.46666666666666667</v>
       </c>
       <c r="F3" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="B4">
-        <f>B3*('Source Data'!$C$3/'Source Data'!$C$2)</f>
+        <f>B3*('Исходные данные'!$D$3/'Исходные данные'!$D$2)</f>
         <v>0.39583333333333331</v>
       </c>
       <c r="C4">
-        <f>C3*('Source Data'!$C$21/'Source Data'!$C$20)</f>
+        <f>C3*('Исходные данные'!$D$21/'Исходные данные'!$D$20)</f>
         <v>0.21111111111111108</v>
       </c>
       <c r="D4">
@@ -2721,19 +2878,19 @@
         <v>-0.46666666666666673</v>
       </c>
       <c r="F4" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B5">
-        <f>'Source Data'!$C$10*'Source Data'!$C$11</f>
+        <f>'Исходные данные'!$D$10*'Исходные данные'!$D$11</f>
         <v>25300</v>
       </c>
       <c r="C5">
-        <f>'Source Data'!$C$28*'Source Data'!$C$29</f>
+        <f>'Исходные данные'!$D$28*'Исходные данные'!$D$29</f>
         <v>75900</v>
       </c>
       <c r="D5">
@@ -2745,19 +2902,19 @@
         <v>2</v>
       </c>
       <c r="F5" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="B6">
-        <f>('Source Data'!$C$9+'Source Data'!$C$10*'Source Data'!$C$11+'Source Data'!$C$14+'Source Data'!$C$12/'Source Data'!$C$13/12)/'Source Data'!$C$8</f>
+        <f>('Исходные данные'!$D$9+'Исходные данные'!$D$10*'Исходные данные'!$D$11+'Исходные данные'!$D$14+'Исходные данные'!$D$12/'Исходные данные'!$D$13/12)/'Исходные данные'!$D$8</f>
         <v>14713.037495700037</v>
       </c>
       <c r="C6">
-        <f>('Source Data'!$C$27+'Source Data'!$C$28*'Source Data'!$C$29+'Source Data'!$C$32+'Source Data'!$C$30/'Source Data'!$C$31/12)/'Source Data'!$C$26</f>
+        <f>('Исходные данные'!$D$27+'Исходные данные'!$D$28*'Исходные данные'!$D$29+'Исходные данные'!$D$32+'Исходные данные'!$D$30/'Исходные данные'!$D$31/12)/'Исходные данные'!$D$26</f>
         <v>15339.662882696941</v>
       </c>
       <c r="D6">
@@ -2769,12 +2926,12 @@
         <v>4.2589804258980429E-2</v>
       </c>
       <c r="F6" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B7">
         <f>B6</f>
@@ -2793,12 +2950,12 @@
         <v>4.2589804258980429E-2</v>
       </c>
       <c r="F7" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="B8">
         <f>TTM!G4</f>
@@ -2817,7 +2974,7 @@
         <v>#N/A</v>
       </c>
       <c r="F8" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2841,36 +2998,36 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="B2">
         <v>0.8125</v>
@@ -2888,15 +3045,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G2" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I2" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B3">
         <v>14713.03749570004</v>
@@ -2914,15 +3071,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G3" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I3" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="B4">
         <v>14713.03749570004</v>
@@ -2940,15 +3097,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G4" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I4" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B5">
         <v>25300</v>
@@ -2966,15 +3123,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G5" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I5" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="B6">
         <v>1424.148606811146</v>
@@ -2992,15 +3149,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G6" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I6" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="B7">
         <v>0.75</v>
@@ -3018,15 +3175,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G7" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I7" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="B8">
         <v>0.85</v>
@@ -3044,32 +3201,32 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G8" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I8" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="F9">
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G9" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="H9" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="I9" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="B10">
         <v>777777.77777777787</v>
@@ -3087,15 +3244,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G10" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I10" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="B11">
         <v>0.59375</v>
@@ -3113,15 +3270,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G11" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I11" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B12">
         <v>0.97435897435897434</v>
@@ -3139,15 +3296,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G12" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I12" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="B13">
         <v>0.75</v>
@@ -3165,15 +3322,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G13" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I13" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="B14">
         <v>2972.1362229102169</v>
@@ -3191,15 +3348,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G14" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I14" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="B15">
         <v>0.39583333333333331</v>
@@ -3217,15 +3374,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G15" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I15" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="B16">
         <v>0.26285941114120442</v>
@@ -3243,15 +3400,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G16" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I16" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B17">
         <v>0.2803468358172122</v>
@@ -3269,15 +3426,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G17" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I17" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="B18">
         <v>1188077.777777778</v>
@@ -3295,15 +3452,15 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G18" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I18" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="B19">
         <v>0.66666666666666663</v>
@@ -3321,10 +3478,10 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="G19" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="I19" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -3344,15 +3501,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="B2">
         <v>0.25</v>
@@ -3360,7 +3517,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="B3">
         <v>0.2</v>
@@ -3368,7 +3525,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="B4">
         <v>0.3</v>
@@ -3376,7 +3533,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="B5">
         <v>0.15</v>
@@ -3384,7 +3541,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="B6">
         <v>0.1</v>
@@ -3412,82 +3569,82 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="B2" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="C2" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="D2" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="E2" t="s">
-        <v>145</v>
+        <v>202</v>
       </c>
       <c r="F2" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="B3" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="C3" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="D3" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="E3" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="F3" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="B4" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="C4" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="D4" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="E4" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="F4" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -3509,70 +3666,70 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>218</v>
       </c>
       <c r="C2" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="D2" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="E2" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="B3" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
       <c r="C3" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="D3" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="E3" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="D4" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
       <c r="E4" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: publish final Harness Log evidence
</commit_message>
<xml_diff>
--- a/1/app/output/ground_truth.xlsx
+++ b/1/app/output/ground_truth.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Economic analysis of knowledge‑intensive industries\1\app\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F6F88E-26FC-4D47-8592-6AB1BC3CA962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A49C96-5C63-45EE-A25E-106DF0E58B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,21 +18,23 @@
     <sheet name="Затраты" sheetId="3" r:id="rId3"/>
     <sheet name="TTM" sheetId="4" r:id="rId4"/>
     <sheet name="Стресс-тест" sheetId="5" r:id="rId5"/>
-    <sheet name="Журнал сверки" sheetId="6" r:id="rId6"/>
-    <sheet name="Структура OPEX" sheetId="7" r:id="rId7"/>
-    <sheet name="Допущения" sheetId="8" r:id="rId8"/>
-    <sheet name="Проблемы данных" sheetId="9" r:id="rId9"/>
+    <sheet name="Сверка Excel–Python" sheetId="6" r:id="rId6"/>
+    <sheet name="Harness Log" sheetId="7" r:id="rId7"/>
+    <sheet name="Структура OPEX" sheetId="8" r:id="rId8"/>
+    <sheet name="Допущения" sheetId="9" r:id="rId9"/>
+    <sheet name="Проблемы данных" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
+    <definedName name="_FilterDatabase" localSheetId="6" hidden="1">'Harness Log'!$A$1:$H$8</definedName>
     <definedName name="_FilterDatabase" localSheetId="3" hidden="1">TTM!$A$1:$H$5</definedName>
-    <definedName name="_FilterDatabase" localSheetId="7" hidden="1">Допущения!$A$1:$F$4</definedName>
-    <definedName name="_FilterDatabase" localSheetId="5" hidden="1">'Журнал сверки'!$A$1:$I$1</definedName>
+    <definedName name="_FilterDatabase" localSheetId="8" hidden="1">Допущения!$A$1:$F$4</definedName>
     <definedName name="_FilterDatabase" localSheetId="2" hidden="1">Затраты!$A$1:$F$7</definedName>
     <definedName name="_FilterDatabase" localSheetId="0" hidden="1">'Исходные данные'!$A$1:$F$37</definedName>
     <definedName name="_FilterDatabase" localSheetId="1" hidden="1">Метрики!$A$1:$F$15</definedName>
-    <definedName name="_FilterDatabase" localSheetId="8" hidden="1">'Проблемы данных'!$A$1:$E$4</definedName>
+    <definedName name="_FilterDatabase" localSheetId="9" hidden="1">'Проблемы данных'!$A$1:$E$4</definedName>
+    <definedName name="_FilterDatabase" localSheetId="5" hidden="1">'Сверка Excel–Python'!$A$1:$I$1</definedName>
     <definedName name="_FilterDatabase" localSheetId="4" hidden="1">'Стресс-тест'!$A$1:$F$8</definedName>
-    <definedName name="_FilterDatabase" localSheetId="6" hidden="1">'Структура OPEX'!$A$1:$B$6</definedName>
+    <definedName name="_FilterDatabase" localSheetId="7" hidden="1">'Структура OPEX'!$A$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
@@ -53,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="287">
   <si>
     <t>Сценарий</t>
   </si>
@@ -607,10 +609,181 @@
     <t>СОВПАДАЕТ</t>
   </si>
   <si>
-    <t>2026-09-14T08:59:36.107726+00:00</t>
+    <t>2026-09-17T10:28:02.400846+00:00</t>
   </si>
   <si>
     <t>Значение Excel недоступно</t>
+  </si>
+  <si>
+    <t>№</t>
+  </si>
+  <si>
+    <t>Этап</t>
+  </si>
+  <si>
+    <t>Запрос к ИИ / задача</t>
+  </si>
+  <si>
+    <t>Сгенерированный или изменённый фрагмент кода</t>
+  </si>
+  <si>
+    <t>Обнаруженная ошибка / галлюцинация</t>
+  </si>
+  <si>
+    <t>Причина</t>
+  </si>
+  <si>
+    <t>Как исправлено</t>
+  </si>
+  <si>
+    <t>Результат повторной проверки</t>
+  </si>
+  <si>
+    <t>Аудит показателей качества</t>
+  </si>
+  <si>
+    <t>Развести FPY и итоговый выход годных</t>
+  </si>
+  <si>
+    <t>fpy = first_pass_good_units / actual_output; final_yield = final_good_units / actual_output</t>
+  </si>
+  <si>
+    <t>FPY и Final Yield могли быть ошибочно приняты за один показатель</t>
+  </si>
+  <si>
+    <t>Итоговый годный объём включает продукцию после переделки</t>
+  </si>
+  <si>
+    <t>Показатели реализованы и раскрыты раздельно</t>
+  </si>
+  <si>
+    <t>Тест подтверждает FPY 75 %, Final Yield 85 %</t>
+  </si>
+  <si>
+    <t>Аудит параметров TTM</t>
+  </si>
+  <si>
+    <t>Сопоставить параметры задания и CSV</t>
+  </si>
+  <si>
+    <t>assignment_ttm = ttm.calculate(delay, 0.10, 0.15, 3.0, window)</t>
+  </si>
+  <si>
+    <t>В задании r=10 %, α=15 %, а в CSV r=12 %, α=18 %</t>
+  </si>
+  <si>
+    <t>Исходные материалы задают разные сценарии</t>
+  </si>
+  <si>
+    <t>Оба сценария рассчитаны и раскрыты отдельно</t>
+  </si>
+  <si>
+    <t>Получены штрафы 26,285941 % и 28,034684 % без подмены параметров</t>
+  </si>
+  <si>
+    <t>Стресс-сценарий TTM</t>
+  </si>
+  <si>
+    <t>Выбрать корректную базовую задержку</t>
+  </si>
+  <si>
+    <t>baseline_stress_ttm = ttm.calculate(comparison.delay[0], 0.10, 0.15, 3.0, window)</t>
+  </si>
+  <si>
+    <t>Pilot CSV содержит задержку 0,5 года, comparison baseline — 0 лет</t>
+  </si>
+  <si>
+    <t>Pilot и сравнительный baseline имеют разное назначение</t>
+  </si>
+  <si>
+    <t>Для стресс-сравнения использован baseline comparison CSV</t>
+  </si>
+  <si>
+    <t>Тест подтверждает изменение штрафа TTM с 0 % до 26,285941 %</t>
+  </si>
+  <si>
+    <t>Аудит ресурсоёмкости</t>
+  </si>
+  <si>
+    <t>Проверить вычислимость массовой ресурсоёмкости</t>
+  </si>
+  <si>
+    <t>mass_intensity = NOT_COMPUTABLE</t>
+  </si>
+  <si>
+    <t>Масса сырья отсутствует, а стоимость не может заменить массу</t>
+  </si>
+  <si>
+    <t>В CSV нет Raw_Material_Mass_kg</t>
+  </si>
+  <si>
+    <t>Метрика помечена НЕ РАССЧИТЫВАЕТСЯ, стоимостной proxy показан отдельно</t>
+  </si>
+  <si>
+    <t>Excel и Python одинаково фиксируют одно невычислимое значение</t>
+  </si>
+  <si>
+    <t>Пересчёт Excel</t>
+  </si>
+  <si>
+    <t>Получить кэшированные результаты формул</t>
+  </si>
+  <si>
+    <t>excel.CalculateFullRebuild(); workbook.Save()</t>
+  </si>
+  <si>
+    <t>openpyxl сохраняет формулы, но не вычисляет их</t>
+  </si>
+  <si>
+    <t>Библиотека не является движком Excel</t>
+  </si>
+  <si>
+    <t>Добавлен реальный пересчёт установленным Microsoft Excel</t>
+  </si>
+  <si>
+    <t>Из кэша прочитаны FPY 0,75, OEE 0,59375 и CPU 14 713,0374957</t>
+  </si>
+  <si>
+    <t>Жизненный цикл COM</t>
+  </si>
+  <si>
+    <t>Исключить сбой освобождения Excel COM</t>
+  </si>
+  <si>
+    <t>subprocess.run([sys.executable, excel_worker.py, workbook_path])</t>
+  </si>
+  <si>
+    <t>Первый интеграционный подход мог завершаться RPC_E_DISCONNECTED</t>
+  </si>
+  <si>
+    <t>COM-прокси переживали закрытие Excel в долгоживущем процессе</t>
+  </si>
+  <si>
+    <t>Пересчёт изолирован в короткоживущем worker-процессе</t>
+  </si>
+  <si>
+    <t>Интеграционный тест завершается без RPC fault и с корректным кэшем</t>
+  </si>
+  <si>
+    <t>Архитектура контрольных журналов</t>
+  </si>
+  <si>
+    <t>Развести журнал реализации и числовую сверку</t>
+  </si>
+  <si>
+    <t>implementation_log_entries и reconciliation_rows</t>
+  </si>
+  <si>
+    <t>Числовая сверка была ошибочно названа Harness Log</t>
+  </si>
+  <si>
+    <t>Два разных типа доказательств использовали одно название</t>
+  </si>
+  <si>
+    <t>Числовая проверка переименована в «Сверка Excel–Python», Harness Log выделен отдельно</t>
+  </si>
+  <si>
+    <t>Отчёты содержат два самостоятельных раздела и восемь обязательных артефактов</t>
   </si>
   <si>
     <t>Категория затрат</t>
@@ -792,12 +965,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -915,7 +1094,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E6C5-4274-8E61-F763DFF8B5D4}"/>
+              <c16:uniqueId val="{00000000-3A75-4F98-B757-E66A9AA88445}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1031,7 +1210,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1062,7 +1241,7 @@
         <xdr:cNvPr id="3" name="Image 2" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2130,6 +2309,91 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="38" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="56" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C2" t="s">
+        <v>276</v>
+      </c>
+      <c r="D2" t="s">
+        <v>277</v>
+      </c>
+      <c r="E2" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B3" t="s">
+        <v>280</v>
+      </c>
+      <c r="C3" t="s">
+        <v>281</v>
+      </c>
+      <c r="D3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E3" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>284</v>
+      </c>
+      <c r="B4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" t="s">
+        <v>281</v>
+      </c>
+      <c r="D4" t="s">
+        <v>285</v>
+      </c>
+      <c r="E4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E4" xr:uid="{00000000-0009-0000-0000-000009000000}"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F15"/>
@@ -3492,6 +3756,234 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
+    <col min="4" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="35" customWidth="1"/>
+    <col min="7" max="7" width="42" customWidth="1"/>
+    <col min="8" max="8" width="38" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>242</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H8" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3501,15 +3993,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>186</v>
+        <v>243</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>187</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>188</v>
+        <v>245</v>
       </c>
       <c r="B2">
         <v>0.25</v>
@@ -3517,7 +4009,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>189</v>
+        <v>246</v>
       </c>
       <c r="B3">
         <v>0.2</v>
@@ -3525,7 +4017,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>190</v>
+        <v>247</v>
       </c>
       <c r="B4">
         <v>0.3</v>
@@ -3533,7 +4025,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>191</v>
+        <v>248</v>
       </c>
       <c r="B5">
         <v>0.15</v>
@@ -3541,21 +4033,21 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>192</v>
+        <v>249</v>
       </c>
       <c r="B6">
         <v>0.1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B6" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <autoFilter ref="A1:B6" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3569,19 +4061,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>250</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>194</v>
+        <v>251</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>195</v>
+        <v>252</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>196</v>
+        <v>253</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>197</v>
+        <v>254</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>180</v>
@@ -3589,151 +4081,66 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>198</v>
+        <v>255</v>
       </c>
       <c r="B2" t="s">
-        <v>199</v>
+        <v>256</v>
       </c>
       <c r="C2" t="s">
-        <v>200</v>
+        <v>257</v>
       </c>
       <c r="D2" t="s">
-        <v>201</v>
+        <v>258</v>
       </c>
       <c r="E2" t="s">
-        <v>202</v>
+        <v>259</v>
       </c>
       <c r="F2" t="s">
-        <v>203</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>204</v>
+        <v>261</v>
       </c>
       <c r="B3" t="s">
-        <v>205</v>
+        <v>262</v>
       </c>
       <c r="C3" t="s">
-        <v>206</v>
+        <v>263</v>
       </c>
       <c r="D3" t="s">
-        <v>207</v>
+        <v>264</v>
       </c>
       <c r="E3" t="s">
-        <v>208</v>
+        <v>265</v>
       </c>
       <c r="F3" t="s">
-        <v>203</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>209</v>
+        <v>266</v>
       </c>
       <c r="B4" t="s">
-        <v>210</v>
+        <v>267</v>
       </c>
       <c r="C4" t="s">
-        <v>211</v>
+        <v>268</v>
       </c>
       <c r="D4" t="s">
-        <v>212</v>
+        <v>269</v>
       </c>
       <c r="E4" t="s">
-        <v>213</v>
+        <v>270</v>
       </c>
       <c r="F4" t="s">
-        <v>203</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="38" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="56" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>217</v>
-      </c>
-      <c r="B2" t="s">
-        <v>218</v>
-      </c>
-      <c r="C2" t="s">
-        <v>219</v>
-      </c>
-      <c r="D2" t="s">
-        <v>220</v>
-      </c>
-      <c r="E2" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>222</v>
-      </c>
-      <c r="B3" t="s">
-        <v>223</v>
-      </c>
-      <c r="C3" t="s">
-        <v>224</v>
-      </c>
-      <c r="D3" t="s">
-        <v>225</v>
-      </c>
-      <c r="E3" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>227</v>
-      </c>
-      <c r="B4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" t="s">
-        <v>224</v>
-      </c>
-      <c r="D4" t="s">
-        <v>228</v>
-      </c>
-      <c r="E4" t="s">
-        <v>229</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E4" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
+  <autoFilter ref="A1:F4" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>